<commit_message>
task 2 & 3 agreement
</commit_message>
<xml_diff>
--- a/results/Image-caption_GT_ VS_Human_Rating.xlsx
+++ b/results/Image-caption_GT_ VS_Human_Rating.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minni\comparative_image_caption\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BB8050-F3A7-41B3-892F-81952DA1BB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15C2A7F-59F8-4510-9F75-430890CE90AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="8964" firstSheet="1" activeTab="1" xr2:uid="{D6321BD8-A525-441C-A5AC-E2373B91F963}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="4" xr2:uid="{D6321BD8-A525-441C-A5AC-E2373B91F963}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression - Task 1" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="49">
   <si>
     <t>Task 1</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>Rater</t>
+  </si>
+  <si>
+    <t>GT_choice</t>
   </si>
 </sst>
 </file>
@@ -2003,7 +2006,7 @@
     <col min="10" max="11" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -2046,8 +2049,11 @@
       <c r="N1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2093,8 +2099,12 @@
         <f>(L2*(L2-1) + M2*(M2-1)) / (COUNTA($D2:$K2) * (COUNTA($D2:$K2) - 1))</f>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O2" t="str">
+        <f t="shared" ref="O2:O11" si="0">IF(B2&gt;C2,"A","B")</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2129,19 +2139,23 @@
         <v>21</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:L11" si="0">COUNTIF($D3:$K3,"A")</f>
+        <f t="shared" ref="L3:L11" si="1">COUNTIF($D3:$K3,"A")</f>
         <v>8</v>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M11" si="1">COUNTIF($D3:$K3,"B")</f>
+        <f t="shared" ref="M3:M11" si="2">COUNTIF($D3:$K3,"B")</f>
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N11" si="2">(L3*(L3-1) + M3*(M3-1)) / (COUNTA($D3:$K3) * (COUNTA($D3:$K3) - 1))</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="shared" ref="N3:N11" si="3">(L3*(L3-1) + M3*(M3-1)) / (COUNTA($D3:$K3) * (COUNTA($D3:$K3) - 1))</f>
+        <v>1</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2176,207 +2190,227 @@
         <v>21</v>
       </c>
       <c r="L4">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="M4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O4" t="str">
         <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="M4">
+      <c r="M5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="0"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="M6">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5">
+        <v>8</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O6" t="str">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="M5">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6">
+        <v>7</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="3"/>
+        <v>0.75</v>
+      </c>
+      <c r="O7" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M6">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="N6">
+      <c r="M8">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J7" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O8" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="M7">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-      <c r="N7">
-        <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="M8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2411,19 +2445,23 @@
         <v>21</v>
       </c>
       <c r="L9">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O9" t="str">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="M9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -2458,19 +2496,23 @@
         <v>21</v>
       </c>
       <c r="L10">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O10" t="str">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="M10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>A</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2505,16 +2547,20 @@
         <v>21</v>
       </c>
       <c r="L11">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="O11" t="str">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="M11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <f t="shared" si="2"/>
-        <v>1</v>
+        <v>A</v>
       </c>
     </row>
     <row r="17" spans="10:15" x14ac:dyDescent="0.3">
@@ -2569,12 +2615,14 @@
   <dimension ref="A1:O18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
     <col min="12" max="12" width="12.77734375" customWidth="1"/>
     <col min="13" max="13" width="13.33203125" customWidth="1"/>
     <col min="14" max="14" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>35</v>
       </c>
@@ -2617,8 +2665,11 @@
       <c r="N1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2664,8 +2715,12 @@
         <f>(L2*(L2-1) + M2*(M2-1)) / (COUNTA($D2:$K2) * (COUNTA($D2:$K2) - 1))</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O2" t="str">
+        <f>IF(B2&gt;C2,"A","B")</f>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2711,8 +2766,12 @@
         <f t="shared" ref="N3:N11" si="2">(L3*(L3-1) + M3*(M3-1)) / (COUNTA($D3:$K3) * (COUNTA($D3:$K3) - 1))</f>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O11" si="3">IF(B3&gt;C3,"A","B")</f>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2758,8 +2817,12 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O4" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -2805,8 +2868,12 @@
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O5" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2852,8 +2919,12 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O6" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2899,8 +2970,12 @@
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O7" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2946,8 +3021,12 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O8" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2993,8 +3072,12 @@
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O9" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -3040,8 +3123,12 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O10" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3086,6 +3173,10 @@
       <c r="N11">
         <f t="shared" si="2"/>
         <v>1</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
       </c>
     </row>
     <row r="17" spans="8:15" x14ac:dyDescent="0.3">
@@ -3290,20 +3381,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ffb1b1c5-72c4-48ac-bba8-4a4e3a1880ef" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ffb1b1c5-72c4-48ac-bba8-4a4e3a1880ef" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3325,14 +3416,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7FAB176-4C42-4DC5-9B33-BCF55F3060F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F323F74F-B6DA-4C5E-B805-085C5F3AAEAF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -3346,4 +3429,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7FAB176-4C42-4DC5-9B33-BCF55F3060F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Organize image-caption GT data into task-specific sheets
</commit_message>
<xml_diff>
--- a/results/Image-caption_GT_ VS_Human_Rating.xlsx
+++ b/results/Image-caption_GT_ VS_Human_Rating.xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minni\comparative_image_caption\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15C2A7F-59F8-4510-9F75-430890CE90AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0B520F-062B-4660-961F-CA842FABA0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="4" xr2:uid="{D6321BD8-A525-441C-A5AC-E2373B91F963}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="7" xr2:uid="{D6321BD8-A525-441C-A5AC-E2373B91F963}"/>
   </bookViews>
   <sheets>
-    <sheet name="Regression - Task 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Inter-Rater (Pearson)" sheetId="4" r:id="rId2"/>
-    <sheet name="Inter-Rater(Spearman)" sheetId="6" r:id="rId3"/>
-    <sheet name="Comparative - Task 2" sheetId="2" r:id="rId4"/>
-    <sheet name="Same_Image -  Task 3 " sheetId="3" r:id="rId5"/>
+    <sheet name="task1" sheetId="7" r:id="rId1"/>
+    <sheet name="task2" sheetId="8" r:id="rId2"/>
+    <sheet name="task3" sheetId="9" r:id="rId3"/>
+    <sheet name="Regression - Task 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Inter-Rater (Pearson)" sheetId="4" r:id="rId5"/>
+    <sheet name="Inter-Rater(Spearman)" sheetId="6" r:id="rId6"/>
+    <sheet name="Comparative - Task 2" sheetId="2" r:id="rId7"/>
+    <sheet name="Same_Image -  Task 3 " sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="152">
   <si>
     <t>Task 1</t>
   </si>
@@ -209,13 +212,322 @@
   </si>
   <si>
     <t>GT_choice</t>
+  </si>
+  <si>
+    <t>Image</t>
+  </si>
+  <si>
+    <t>Caption</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000404780.jpg</t>
+  </si>
+  <si>
+    <t>a group of people that are on the beach .</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000511594.jpg</t>
+  </si>
+  <si>
+    <t>a woman in a red jacket is standing next to a sign .</t>
+  </si>
+  <si>
+    <t>A man in a black jacket is walking down a hill.</t>
+  </si>
+  <si>
+    <t>A man on a motorcycle going down the street.</t>
+  </si>
+  <si>
+    <t>An apple sitting on top of a laptop.</t>
+  </si>
+  <si>
+    <t>A man with some suitcases on the street.</t>
+  </si>
+  <si>
+    <t>A large building with a clock tower is lit up at night.</t>
+  </si>
+  <si>
+    <t>People walking down the street in the rain.</t>
+  </si>
+  <si>
+    <t>A double oven mounted inside of a yellow wall.</t>
+  </si>
+  <si>
+    <t> A group of people standing next to each other.</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000063563.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000421370.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000038252.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000393578.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000053139.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000555002.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000192656.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000323799.jpg</t>
+  </si>
+  <si>
+    <t>A table and chairs sit on a grassy walkway, with a pitcher</t>
+  </si>
+  <si>
+    <t>Orange construction equipment sitting on the side of the road</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000395865.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000344844.jpg</t>
+  </si>
+  <si>
+    <t>A cat laying on the ground next to a person</t>
+  </si>
+  <si>
+    <t>A man is riding a bike in the snow.</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000501382.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000030504.jpg</t>
+  </si>
+  <si>
+    <t>A man standing in front of a brick wall.</t>
+  </si>
+  <si>
+    <t>A laptop next to two computers, keyboards and some mouses.</t>
+  </si>
+  <si>
+    <t>A black and white picture of vehicles and people in the street.</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000301347.jpg</t>
+  </si>
+  <si>
+    <t>a dog is standing in the snow with a large stick .</t>
+  </si>
+  <si>
+    <t>A large tree with a lot of decorations on it.</t>
+  </si>
+  <si>
+    <t>Two burritos on a plate with a spoon next to a pack of cigarettes.</t>
+  </si>
+  <si>
+    <t>A bathroom is shown, with a urinal and a bidet.</t>
+  </si>
+  <si>
+    <t> A dog is laying on the grass with a leash.</t>
+  </si>
+  <si>
+    <t>A car is parked in front of a building</t>
+  </si>
+  <si>
+    <t>A squirrel is standing on a rock with a rope.</t>
+  </si>
+  <si>
+    <t>A herd of sheep in an open snowy field.</t>
+  </si>
+  <si>
+    <t>A computer screen is displayed with a lot of books.</t>
+  </si>
+  <si>
+    <t>A bird themed clock sitting inside of a green box.</t>
+  </si>
+  <si>
+    <t>A young man holding a skateboard while wearing head phones.</t>
+  </si>
+  <si>
+    <t>A man standing next to a cart filled with bananas.</t>
+  </si>
+  <si>
+    <t>This is a toy microwave and toy foods.</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000488069.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000524245.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000222548.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000043555.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000573565.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000361172.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000221693.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000290798.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000391029.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000393928.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000025846.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000386193.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000372494.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000093068.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000356236.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>A cow walking in front of a red car</t>
+  </si>
+  <si>
+    <t>A decorated truck is parked at a curb near a building.</t>
+  </si>
+  <si>
+    <t>A truck with graffiti on the side of it</t>
+  </si>
+  <si>
+    <t>Mom gives her daughter a lesson in using her baseball glove.</t>
+  </si>
+  <si>
+    <t>A group of young people playing a game of baseball</t>
+  </si>
+  <si>
+    <t>An electric tower in front of buildings on the road.</t>
+  </si>
+  <si>
+    <t>A train that is sitting on the side of a road</t>
+  </si>
+  <si>
+    <t>A  girl in a purple shirt holding a backpack.</t>
+  </si>
+  <si>
+    <t>A girl smiles while holding a baseball glove.</t>
+  </si>
+  <si>
+    <t>A close up of a house phone showing only the numbers in focus.</t>
+  </si>
+  <si>
+    <t>A remote control sitting on top of a keyboard</t>
+  </si>
+  <si>
+    <t>A blue umbrella sitting in the ground next to a fence</t>
+  </si>
+  <si>
+    <t>A fire hydrant with a blue jacket on top of it.</t>
+  </si>
+  <si>
+    <t>A bathroom with a sink and a mirror.</t>
+  </si>
+  <si>
+    <t>A public bathroom with a white sink and sign regarding dirty hands.</t>
+  </si>
+  <si>
+    <t>A trio of dogs sitting in their owner's lap in a red convertible.</t>
+  </si>
+  <si>
+    <t>A woman and her dog in the back of a car</t>
+  </si>
+  <si>
+    <t>Naan bread, soup, and a drink are served on a cafeteria tray.</t>
+  </si>
+  <si>
+    <t>A plate with a sandwich and a cup of soup</t>
+  </si>
+  <si>
+    <t>Cows walking down a street near a tour bus. </t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000416385.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000521052.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000185240.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000006789.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000162415.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000570242.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000005437.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000188733.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000407286.jpg</t>
+  </si>
+  <si>
+    <t>http://images.cocodataset.org/val2014/COCO_val2014_000000085481.jpg</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Majority_Vote</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,8 +555,33 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF32363A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -254,6 +591,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -341,7 +684,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -363,6 +706,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -702,6 +1052,760 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C3700B0-F235-4E67-9553-F71FD08F60BB}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="61" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11">
+        <v>4.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43AE4EAA-E546-42B0-A1F8-01FEFD3E7EF4}">
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="17"/>
+      <c r="B3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="17"/>
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="17"/>
+      <c r="B9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="17"/>
+      <c r="B11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="17"/>
+      <c r="B15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="17"/>
+      <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="17"/>
+      <c r="B19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="17"/>
+      <c r="B21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G24" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38A5F46E-8018-4704-8A9F-DCA230CB137B}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2">
+        <v>4.74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D15">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D21">
+        <v>4.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ECE4A2F-5696-4BC6-80B6-FD2C6A94C8FD}">
   <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -768,7 +1872,7 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="C2">
         <v>3</v>
@@ -795,16 +1899,16 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <f t="shared" ref="K2:K11" si="0" xml:space="preserve"> ROUND(AVERAGE(C2:I2),0)</f>
-        <v>2</v>
+        <f>AVERAGE(C2:J2)</f>
+        <v>2.125</v>
       </c>
       <c r="L2" t="str">
         <f>IF(MAX(C2:J2)=MIN(C2:J2),"All Same","Different")</f>
         <v>Different</v>
       </c>
       <c r="M2" t="str" cm="1">
-        <f t="array" ref="M2">IF(MAX(COUNTIF($C2:$J2,$C2:$J2))&gt;=3,"Majority Same","Different")</f>
-        <v>Majority Same</v>
+        <f t="array" ref="M2">IF(MAX(COUNTIF($C2:$J2,$C2:$J2))&gt;=5,"Majority Same","Different")</f>
+        <v>Different</v>
       </c>
       <c r="N2">
         <f>_xlfn.STDEV.S(C2:J2)</f>
@@ -812,15 +1916,15 @@
       </c>
       <c r="O2">
         <f>ABS(B2 - K2)</f>
-        <v>0</v>
+        <v>0.27499999999999991</v>
       </c>
       <c r="P2" s="1">
         <f>_xlfn.RANK.AVG(B2,$B$2:$B$11,0)</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="Q2" s="1">
         <f>_xlfn.RANK.AVG(K2,$K$2:$K$11,0)</f>
-        <v>5.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
@@ -828,7 +1932,7 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -855,7 +1959,7 @@
         <v>1</v>
       </c>
       <c r="K3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="K3:K11" si="0">AVERAGE(C3:J3)</f>
         <v>1</v>
       </c>
       <c r="L3" t="str">
@@ -863,7 +1967,7 @@
         <v>All Same</v>
       </c>
       <c r="M3" t="str" cm="1">
-        <f t="array" ref="M3">IF(MAX(COUNTIF($C3:$J3,$C3:$J3))&gt;=3,"Majority Same","Different")</f>
+        <f t="array" ref="M3">IF(MAX(COUNTIF($C3:$J3,$C3:$J3))&gt;=5,"Majority Same","Different")</f>
         <v>Majority Same</v>
       </c>
       <c r="N3">
@@ -872,15 +1976,15 @@
       </c>
       <c r="O3">
         <f t="shared" ref="O3:O11" si="3">ABS(B3 - K3)</f>
-        <v>0</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="P3" s="1">
         <f t="shared" ref="P3:P11" si="4">_xlfn.RANK.AVG(B3,$B$2:$B$11,0)</f>
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="Q3" s="1">
         <f t="shared" ref="Q3:Q11" si="5">_xlfn.RANK.AVG(K3,$K$2:$K$11,0)</f>
-        <v>9</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
@@ -916,15 +2020,15 @@
       </c>
       <c r="K4">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1.875</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="1"/>
         <v>Different</v>
       </c>
       <c r="M4" t="str" cm="1">
-        <f t="array" ref="M4">IF(MAX(COUNTIF($C4:$J4,$C4:$J4))&gt;=3,"Majority Same","Different")</f>
-        <v>Majority Same</v>
+        <f t="array" ref="M4">IF(MAX(COUNTIF($C4:$J4,$C4:$J4))&gt;=5,"Majority Same","Different")</f>
+        <v>Different</v>
       </c>
       <c r="N4">
         <f t="shared" si="2"/>
@@ -932,15 +2036,15 @@
       </c>
       <c r="O4">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="P4" s="1">
         <f t="shared" si="4"/>
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="1">
         <f t="shared" si="5"/>
-        <v>5.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -976,14 +2080,14 @@
       </c>
       <c r="K5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="1"/>
         <v>Different</v>
       </c>
       <c r="M5" t="str" cm="1">
-        <f t="array" ref="M5">IF(MAX(COUNTIF($C5:$J5,$C5:$J5))&gt;=3,"Majority Same","Different")</f>
+        <f t="array" ref="M5">IF(MAX(COUNTIF($C5:$J5,$C5:$J5))&gt;=5,"Majority Same","Different")</f>
         <v>Majority Same</v>
       </c>
       <c r="N5">
@@ -992,11 +2096,11 @@
       </c>
       <c r="O5">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="P5" s="1">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="1">
         <f t="shared" si="5"/>
@@ -1036,15 +2140,15 @@
       </c>
       <c r="K6">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2.375</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="1"/>
         <v>Different</v>
       </c>
       <c r="M6" t="str" cm="1">
-        <f t="array" ref="M6">IF(MAX(COUNTIF($C6:$J6,$C6:$J6))&gt;=3,"Majority Same","Different")</f>
-        <v>Majority Same</v>
+        <f t="array" ref="M6">IF(MAX(COUNTIF($C6:$J6,$C6:$J6))&gt;=5,"Majority Same","Different")</f>
+        <v>Different</v>
       </c>
       <c r="N6">
         <f t="shared" si="2"/>
@@ -1052,15 +2156,15 @@
       </c>
       <c r="O6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="P6" s="1">
         <f t="shared" si="4"/>
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="1">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
@@ -1068,7 +2172,7 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
@@ -1096,15 +2200,15 @@
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>2.375</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="1"/>
         <v>Different</v>
       </c>
       <c r="M7" t="str" cm="1">
-        <f t="array" ref="M7">IF(MAX(COUNTIF($C7:$J7,$C7:$J7))&gt;=3,"Majority Same","Different")</f>
-        <v>Majority Same</v>
+        <f t="array" ref="M7">IF(MAX(COUNTIF($C7:$J7,$C7:$J7))&gt;=5,"Majority Same","Different")</f>
+        <v>Different</v>
       </c>
       <c r="N7">
         <f t="shared" si="2"/>
@@ -1112,7 +2216,7 @@
       </c>
       <c r="O7">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0.375</v>
       </c>
       <c r="P7" s="1">
         <f t="shared" si="4"/>
@@ -1120,7 +2224,7 @@
       </c>
       <c r="Q7" s="1">
         <f t="shared" si="5"/>
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
@@ -1128,7 +2232,7 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
@@ -1156,14 +2260,14 @@
       </c>
       <c r="K8">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="1"/>
         <v>Different</v>
       </c>
       <c r="M8" t="str" cm="1">
-        <f t="array" ref="M8">IF(MAX(COUNTIF($C8:$J8,$C8:$J8))&gt;=3,"Majority Same","Different")</f>
+        <f t="array" ref="M8">IF(MAX(COUNTIF($C8:$J8,$C8:$J8))&gt;=5,"Majority Same","Different")</f>
         <v>Majority Same</v>
       </c>
       <c r="N8">
@@ -1172,15 +2276,15 @@
       </c>
       <c r="O8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="P8" s="1">
         <f t="shared" si="4"/>
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="1">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
@@ -1188,7 +2292,7 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
@@ -1223,8 +2327,8 @@
         <v>Different</v>
       </c>
       <c r="M9" t="str" cm="1">
-        <f t="array" ref="M9">IF(MAX(COUNTIF($C9:$J9,$C9:$J9))&gt;=3,"Majority Same","Different")</f>
-        <v>Majority Same</v>
+        <f t="array" ref="M9">IF(MAX(COUNTIF($C9:$J9,$C9:$J9))&gt;=5,"Majority Same","Different")</f>
+        <v>Different</v>
       </c>
       <c r="N9">
         <f t="shared" si="2"/>
@@ -1232,7 +2336,7 @@
       </c>
       <c r="O9">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="P9" s="1">
         <f t="shared" si="4"/>
@@ -1240,7 +2344,7 @@
       </c>
       <c r="Q9" s="1">
         <f t="shared" si="5"/>
-        <v>5.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1283,7 +2387,7 @@
         <v>All Same</v>
       </c>
       <c r="M10" t="str" cm="1">
-        <f t="array" ref="M10">IF(MAX(COUNTIF($C10:$J10,$C10:$J10))&gt;=3,"Majority Same","Different")</f>
+        <f t="array" ref="M10">IF(MAX(COUNTIF($C10:$J10,$C10:$J10))&gt;=5,"Majority Same","Different")</f>
         <v>Majority Same</v>
       </c>
       <c r="N10">
@@ -1296,11 +2400,11 @@
       </c>
       <c r="P10" s="1">
         <f t="shared" si="4"/>
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="Q10" s="1">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
@@ -1308,7 +2412,7 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="C11" s="1">
         <v>5</v>
@@ -1343,7 +2447,7 @@
         <v>All Same</v>
       </c>
       <c r="M11" t="str" cm="1">
-        <f t="array" ref="M11">IF(MAX(COUNTIF($C11:$J11,$C11:$J11))&gt;=3,"Majority Same","Different")</f>
+        <f t="array" ref="M11">IF(MAX(COUNTIF($C11:$J11,$C11:$J11))&gt;=5,"Majority Same","Different")</f>
         <v>Majority Same</v>
       </c>
       <c r="N11">
@@ -1352,11 +2456,11 @@
       </c>
       <c r="O11">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P11" s="1">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="Q11" s="1">
         <f t="shared" si="5"/>
@@ -1379,7 +2483,7 @@
       </c>
       <c r="M12">
         <f>COUNTIF($M$2:$M$11,"Majority Same")/COUNTA($A$2:$A$11)</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N12">
         <f>AVERAGE(N2:N11)</f>
@@ -1391,11 +2495,11 @@
       </c>
       <c r="S12" s="11">
         <f>CORREL(P2:P11,Q2:Q11)</f>
-        <v>0.77888212966185566</v>
+        <v>0.90826112777287393</v>
       </c>
       <c r="T12" s="12">
         <f>CORREL(B2:B11,K2:K11)</f>
-        <v>0.86732843315220731</v>
+        <v>0.93120323286029272</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
@@ -1407,7 +2511,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7594C4C8-047F-442C-86A8-624F63CB5AEB}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1476,7 +2580,7 @@
       <c r="I2">
         <v>0.64168899999999995</v>
       </c>
-      <c r="J2" s="13">
+      <c r="J2" s="18">
         <f>AVERAGE(C2:H2, D3:H3, E4:H4, F5:H5, G6:H6, H7)</f>
         <v>0.66876109523809535</v>
       </c>
@@ -1509,7 +2613,7 @@
       <c r="I3">
         <v>0.55405099999999996</v>
       </c>
-      <c r="J3" s="13"/>
+      <c r="J3" s="18"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -1539,7 +2643,7 @@
       <c r="I4">
         <v>0.47711900000000002</v>
       </c>
-      <c r="J4" s="13"/>
+      <c r="J4" s="18"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1569,7 +2673,7 @@
       <c r="I5">
         <v>0.43732900000000002</v>
       </c>
-      <c r="J5" s="13"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -1599,7 +2703,7 @@
       <c r="I6">
         <v>0.65330500000000002</v>
       </c>
-      <c r="J6" s="13"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -1629,7 +2733,7 @@
       <c r="I7">
         <v>0.72374700000000003</v>
       </c>
-      <c r="J7" s="13"/>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -1659,7 +2763,7 @@
       <c r="I8">
         <v>0.78825299999999998</v>
       </c>
-      <c r="J8" s="13"/>
+      <c r="J8" s="18"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1689,7 +2793,7 @@
       <c r="I9">
         <v>1</v>
       </c>
-      <c r="J9" s="13"/>
+      <c r="J9" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1699,7 +2803,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08CD1F2B-6FE7-4BC8-BEB8-F8F3A1656A9D}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1767,7 +2871,7 @@
       <c r="I2" s="4">
         <v>0.54870300000000005</v>
       </c>
-      <c r="J2" s="14">
+      <c r="J2" s="19">
         <f>AVERAGE(
     C2:I2,
     D3:I3,
@@ -1807,7 +2911,7 @@
       <c r="I3" s="4">
         <v>0.39578000000000002</v>
       </c>
-      <c r="J3" s="14"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -1837,7 +2941,7 @@
       <c r="I4" s="4">
         <v>0.46880699999999997</v>
       </c>
-      <c r="J4" s="14"/>
+      <c r="J4" s="19"/>
     </row>
     <row r="5" spans="1:10" ht="15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -1867,7 +2971,7 @@
       <c r="I5" s="4">
         <v>0.36983500000000002</v>
       </c>
-      <c r="J5" s="14"/>
+      <c r="J5" s="19"/>
     </row>
     <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -1897,7 +3001,7 @@
       <c r="I6" s="1">
         <v>0.40662500000000001</v>
       </c>
-      <c r="J6" s="14"/>
+      <c r="J6" s="19"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -1995,18 +3099,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DECC0E63-D9F8-4606-9CC9-8F89AD470AD7}">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="21.109375" customWidth="1"/>
     <col min="10" max="11" width="19.33203125" customWidth="1"/>
+    <col min="16" max="16" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -2017,28 +3122,28 @@
         <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>143</v>
       </c>
       <c r="F1" t="s">
-        <v>44</v>
+        <v>144</v>
       </c>
       <c r="G1" t="s">
-        <v>45</v>
+        <v>145</v>
       </c>
       <c r="H1" t="s">
-        <v>4</v>
+        <v>146</v>
       </c>
       <c r="I1" t="s">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="J1" t="s">
-        <v>6</v>
+        <v>148</v>
       </c>
       <c r="K1" t="s">
-        <v>46</v>
+        <v>149</v>
       </c>
       <c r="L1" t="s">
         <v>36</v>
@@ -2052,16 +3157,22 @@
       <c r="O1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q1" s="16" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
@@ -2103,16 +3214,19 @@
         <f t="shared" ref="O2:O11" si="0">IF(B2&gt;C2,"A","B")</f>
         <v>B</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P2">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D3" t="s">
         <v>21</v>
@@ -2154,13 +3268,16 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2205,8 +3322,11 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -2256,8 +3376,11 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2265,7 +3388,7 @@
         <v>2</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -2307,8 +3430,11 @@
         <f t="shared" si="0"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2358,8 +3484,11 @@
         <f t="shared" si="0"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P7">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2409,8 +3538,11 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2418,7 +3550,7 @@
         <v>5</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -2460,16 +3592,19 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -2511,16 +3646,19 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -2562,8 +3700,11 @@
         <f t="shared" si="0"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="17" spans="10:15" x14ac:dyDescent="0.3">
+      <c r="P11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J17" s="5" t="s">
         <v>39</v>
       </c>
@@ -2580,8 +3721,9 @@
       <c r="O17" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="18" spans="10:15" x14ac:dyDescent="0.3">
+      <c r="P17" s="5"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J18" s="5">
         <f>AVERAGE($N$2:$N$11)</f>
         <v>0.95</v>
@@ -2603,16 +3745,109 @@
         <f>(J18 - N18)/(1 - N18)</f>
         <v>0.87460815047021934</v>
       </c>
+      <c r="P18" s="5"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B24" s="17"/>
+      <c r="D24" s="14"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B25" s="17"/>
+      <c r="D25" s="14"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B26" s="17"/>
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B27" s="17"/>
+      <c r="D27" s="14"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B28" s="17"/>
+      <c r="D28" s="14"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B29" s="17"/>
+      <c r="D29" s="14"/>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B30" s="17"/>
+      <c r="D30" s="14"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B31" s="17"/>
+      <c r="D31" s="15"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B32" s="17"/>
+      <c r="D32" s="14"/>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B33" s="17"/>
+      <c r="D33" s="14"/>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B34" s="17"/>
+      <c r="D34" s="14"/>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="17"/>
+      <c r="D35" s="14"/>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="17"/>
+      <c r="D36" s="14"/>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B37" s="17"/>
+      <c r="D37" s="14"/>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="17"/>
+      <c r="D38" s="14"/>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B39" s="17"/>
+      <c r="D39" s="14"/>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B40" s="17"/>
+      <c r="D40" s="14"/>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B41" s="17"/>
+      <c r="D41" s="14"/>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B42" s="17"/>
+      <c r="D42" s="14"/>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="17"/>
+      <c r="D43" s="14"/>
     </row>
   </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7547234D-7E4C-441D-9FFB-8E4230BDAB6A}">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.88671875" customWidth="1"/>
@@ -2622,7 +3857,7 @@
     <col min="14" max="14" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>35</v>
       </c>
@@ -2633,28 +3868,28 @@
         <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>143</v>
       </c>
       <c r="F1" t="s">
-        <v>44</v>
+        <v>144</v>
       </c>
       <c r="G1" t="s">
-        <v>45</v>
+        <v>145</v>
       </c>
       <c r="H1" t="s">
-        <v>4</v>
+        <v>146</v>
       </c>
       <c r="I1" t="s">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="J1" t="s">
-        <v>6</v>
+        <v>148</v>
       </c>
       <c r="K1" t="s">
-        <v>46</v>
+        <v>149</v>
       </c>
       <c r="L1" t="s">
         <v>36</v>
@@ -2668,16 +3903,19 @@
       <c r="O1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>4.74</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="D2" t="s">
         <v>21</v>
@@ -2719,8 +3957,11 @@
         <f>IF(B2&gt;C2,"A","B")</f>
         <v>A</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -2728,7 +3969,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -2770,16 +4011,19 @@
         <f t="shared" ref="O3:O11" si="3">IF(B3&gt;C3,"A","B")</f>
         <v>A</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -2821,16 +4065,19 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -2872,16 +4119,19 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -2923,16 +4173,19 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P6">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -2974,16 +4227,19 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -3025,8 +4281,11 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P8">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -3034,7 +4293,7 @@
         <v>3</v>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -3076,8 +4335,11 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P9">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -3085,7 +4347,7 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -3127,16 +4389,19 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -3178,8 +4443,11 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="17" spans="8:15" x14ac:dyDescent="0.3">
+      <c r="P11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="3:15" x14ac:dyDescent="0.3">
       <c r="H17" s="5" t="s">
         <v>39</v>
       </c>
@@ -3199,7 +4467,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="8:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:15" x14ac:dyDescent="0.3">
       <c r="H18" s="5">
         <f>AVERAGE($N$2:$N$11)</f>
         <v>0.9</v>
@@ -3224,7 +4492,130 @@
         <v>0.77207977207977208</v>
       </c>
     </row>
+    <row r="25" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="14"/>
+    </row>
+    <row r="26" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="14"/>
+    </row>
+    <row r="27" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="14"/>
+    </row>
+    <row r="28" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="14"/>
+    </row>
+    <row r="29" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="14"/>
+    </row>
+    <row r="30" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="14"/>
+    </row>
+    <row r="31" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="14"/>
+    </row>
+    <row r="32" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="14"/>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="14"/>
+    </row>
+    <row r="34" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="14"/>
+    </row>
+    <row r="35" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="14"/>
+    </row>
+    <row r="36" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="14"/>
+    </row>
+    <row r="37" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="14"/>
+    </row>
+    <row r="38" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="14"/>
+    </row>
+    <row r="39" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="14"/>
+    </row>
+    <row r="40" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="14"/>
+    </row>
+    <row r="41" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="14"/>
+    </row>
+    <row r="42" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="14"/>
+    </row>
+    <row r="43" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="14"/>
+    </row>
+    <row r="44" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="14"/>
+    </row>
   </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3381,20 +4772,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ffb1b1c5-72c4-48ac-bba8-4a4e3a1880ef" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ffb1b1c5-72c4-48ac-bba8-4a4e3a1880ef" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3416,6 +4807,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7FAB176-4C42-4DC5-9B33-BCF55F3060F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F323F74F-B6DA-4C5E-B805-085C5F3AAEAF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -3429,12 +4828,4 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7FAB176-4C42-4DC5-9B33-BCF55F3060F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>